<commit_message>
Trim Notes column to bare NV license number
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LMPr6MDgEjTi5HVnUn4QyW
</commit_message>
<xml_diff>
--- a/CPBN_list_Active.xlsx
+++ b/CPBN_list_Active.xlsx
@@ -872,7 +872,7 @@
       <c r="AD4" s="2" t="inlineStr"/>
       <c r="AE4" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00958; disciplinary action on record; NV lic #B00521</t>
+          <t>NV lic #B00958</t>
         </is>
       </c>
     </row>
@@ -2734,7 +2734,7 @@
       <c r="AD26" s="2" t="inlineStr"/>
       <c r="AE26" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01660; NV lic #B00462</t>
+          <t>NV lic #B01660</t>
         </is>
       </c>
     </row>
@@ -4248,7 +4248,7 @@
       <c r="AD44" s="2" t="inlineStr"/>
       <c r="AE44" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01400; disciplinary action on record</t>
+          <t>NV lic #B01400</t>
         </is>
       </c>
     </row>
@@ -4843,7 +4843,7 @@
       <c r="AD51" s="2" t="inlineStr"/>
       <c r="AE51" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01933; NV lic #B00681</t>
+          <t>NV lic #B01933</t>
         </is>
       </c>
     </row>
@@ -5098,7 +5098,7 @@
       <c r="AD54" s="2" t="inlineStr"/>
       <c r="AE54" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02067; NV lic #B0988</t>
+          <t>NV lic #B02067</t>
         </is>
       </c>
     </row>
@@ -5353,7 +5353,7 @@
       <c r="AD57" s="2" t="inlineStr"/>
       <c r="AE57" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01437; NV lic #B01521; NV lic #B00190</t>
+          <t>NV lic #B01437</t>
         </is>
       </c>
     </row>
@@ -5774,7 +5774,7 @@
       <c r="AD62" s="2" t="inlineStr"/>
       <c r="AE62" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02007; disciplinary action on record</t>
+          <t>NV lic #B02007</t>
         </is>
       </c>
     </row>
@@ -5944,7 +5944,7 @@
       <c r="AD64" s="2" t="inlineStr"/>
       <c r="AE64" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01588; disciplinary action on record</t>
+          <t>NV lic #B01588</t>
         </is>
       </c>
     </row>
@@ -6280,7 +6280,7 @@
       <c r="AD68" s="2" t="inlineStr"/>
       <c r="AE68" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00523; disciplinary action on record</t>
+          <t>NV lic #B00523</t>
         </is>
       </c>
     </row>
@@ -7041,7 +7041,7 @@
       <c r="AD77" s="2" t="inlineStr"/>
       <c r="AE77" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01929; disciplinary action on record; NV lic #B01652</t>
+          <t>NV lic #B01929</t>
         </is>
       </c>
     </row>
@@ -7798,7 +7798,7 @@
       <c r="AD86" s="2" t="inlineStr"/>
       <c r="AE86" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00917; disciplinary action on record</t>
+          <t>NV lic #B00917</t>
         </is>
       </c>
     </row>
@@ -8988,7 +8988,7 @@
       <c r="AD100" s="2" t="inlineStr"/>
       <c r="AE100" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00368; disciplinary action on record; NV lic #B01825</t>
+          <t>NV lic #B00368</t>
         </is>
       </c>
     </row>
@@ -9158,7 +9158,7 @@
       <c r="AD102" s="2" t="inlineStr"/>
       <c r="AE102" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01302; NV lic #B01039; NV lic #B00852</t>
+          <t>NV lic #B01302</t>
         </is>
       </c>
     </row>
@@ -9409,7 +9409,7 @@
       <c r="AD105" s="2" t="inlineStr"/>
       <c r="AE105" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00753; disciplinary action on record</t>
+          <t>NV lic #B00753</t>
         </is>
       </c>
     </row>
@@ -9660,7 +9660,7 @@
       <c r="AD108" s="2" t="inlineStr"/>
       <c r="AE108" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01219; disciplinary action on record; NV lic #B00460; NV lic #B01511</t>
+          <t>NV lic #B01219</t>
         </is>
       </c>
     </row>
@@ -10935,7 +10935,7 @@
       <c r="AD123" s="2" t="inlineStr"/>
       <c r="AE123" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00586; disciplinary action on record</t>
+          <t>NV lic #B00586</t>
         </is>
       </c>
     </row>
@@ -11190,7 +11190,7 @@
       <c r="AD126" s="2" t="inlineStr"/>
       <c r="AE126" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00757; NV lic #B01867</t>
+          <t>NV lic #B00757</t>
         </is>
       </c>
     </row>
@@ -11445,7 +11445,7 @@
       <c r="AD129" s="2" t="inlineStr"/>
       <c r="AE129" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01509; NV lic #B00442</t>
+          <t>NV lic #B01509</t>
         </is>
       </c>
     </row>
@@ -13315,7 +13315,7 @@
       <c r="AD151" s="2" t="inlineStr"/>
       <c r="AE151" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01341; disciplinary action on record</t>
+          <t>NV lic #B01341</t>
         </is>
       </c>
     </row>
@@ -13825,7 +13825,7 @@
       <c r="AD157" s="2" t="inlineStr"/>
       <c r="AE157" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00376; disciplinary action on record</t>
+          <t>NV lic #B00376</t>
         </is>
       </c>
     </row>
@@ -15780,7 +15780,7 @@
       <c r="AD180" s="2" t="inlineStr"/>
       <c r="AE180" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01985; NV lic #B00255</t>
+          <t>NV lic #B01985</t>
         </is>
       </c>
     </row>
@@ -17476,7 +17476,7 @@
       <c r="AD200" s="2" t="inlineStr"/>
       <c r="AE200" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01937; NV lic #B00184</t>
+          <t>NV lic #B01937</t>
         </is>
       </c>
     </row>
@@ -18156,7 +18156,7 @@
       <c r="AD208" s="2" t="inlineStr"/>
       <c r="AE208" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01047; disciplinary action on record</t>
+          <t>NV lic #B01047</t>
         </is>
       </c>
     </row>
@@ -20706,7 +20706,7 @@
       <c r="AD238" s="2" t="inlineStr"/>
       <c r="AE238" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00861; disciplinary action on record</t>
+          <t>NV lic #B00861</t>
         </is>
       </c>
     </row>
@@ -20876,7 +20876,7 @@
       <c r="AD240" s="2" t="inlineStr"/>
       <c r="AE240" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00220; NV lic #B00496</t>
+          <t>NV lic #B00220</t>
         </is>
       </c>
     </row>
@@ -21556,7 +21556,7 @@
       <c r="AD248" s="2" t="inlineStr"/>
       <c r="AE248" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01464; disciplinary action on record</t>
+          <t>NV lic #B01464</t>
         </is>
       </c>
     </row>
@@ -22831,7 +22831,7 @@
       <c r="AD263" s="2" t="inlineStr"/>
       <c r="AE263" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01793; NV lic #B01878; NV lic #B00634</t>
+          <t>NV lic #B01793</t>
         </is>
       </c>
     </row>
@@ -23596,7 +23596,7 @@
       <c r="AD272" s="2" t="inlineStr"/>
       <c r="AE272" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01662; NV lic #B01528</t>
+          <t>NV lic #B01662</t>
         </is>
       </c>
     </row>
@@ -24191,7 +24191,7 @@
       <c r="AD279" s="2" t="inlineStr"/>
       <c r="AE279" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00617; disciplinary action on record</t>
+          <t>NV lic #B00617</t>
         </is>
       </c>
     </row>
@@ -24956,7 +24956,7 @@
       <c r="AD288" s="2" t="inlineStr"/>
       <c r="AE288" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00158; disciplinary action on record</t>
+          <t>NV lic #B00158</t>
         </is>
       </c>
     </row>
@@ -25381,7 +25381,7 @@
       <c r="AD293" s="2" t="inlineStr"/>
       <c r="AE293" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00846; disciplinary action on record</t>
+          <t>NV lic #B00846</t>
         </is>
       </c>
     </row>
@@ -25466,7 +25466,7 @@
       <c r="AD294" s="2" t="inlineStr"/>
       <c r="AE294" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00745; disciplinary action on record</t>
+          <t>NV lic #B00745</t>
         </is>
       </c>
     </row>
@@ -26826,7 +26826,7 @@
       <c r="AD310" s="2" t="inlineStr"/>
       <c r="AE310" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00474; NV lic #B00830</t>
+          <t>NV lic #B00474</t>
         </is>
       </c>
     </row>
@@ -28781,7 +28781,7 @@
       <c r="AD333" s="2" t="inlineStr"/>
       <c r="AE333" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01795; NV lic #B00109</t>
+          <t>NV lic #B01795</t>
         </is>
       </c>
     </row>
@@ -28951,7 +28951,7 @@
       <c r="AD335" s="2" t="inlineStr"/>
       <c r="AE335" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01383; disciplinary action on record</t>
+          <t>NV lic #B01383</t>
         </is>
       </c>
     </row>
@@ -29206,7 +29206,7 @@
       <c r="AD338" s="2" t="inlineStr"/>
       <c r="AE338" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00187; disciplinary action on record</t>
+          <t>NV lic #B00187</t>
         </is>
       </c>
     </row>
@@ -29291,7 +29291,7 @@
       <c r="AD339" s="2" t="inlineStr"/>
       <c r="AE339" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01034; disciplinary action on record</t>
+          <t>NV lic #B01034</t>
         </is>
       </c>
     </row>
@@ -30141,7 +30141,7 @@
       <c r="AD349" s="2" t="inlineStr"/>
       <c r="AE349" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00648; disciplinary action on record</t>
+          <t>NV lic #B00648</t>
         </is>
       </c>
     </row>
@@ -30906,7 +30906,7 @@
       <c r="AD358" s="2" t="inlineStr"/>
       <c r="AE358" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01537; NV lic #B00751</t>
+          <t>NV lic #B01537</t>
         </is>
       </c>
     </row>
@@ -31246,7 +31246,7 @@
       <c r="AD362" s="2" t="inlineStr"/>
       <c r="AE362" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00705; disciplinary action on record; NV lic #B00293</t>
+          <t>NV lic #B00705</t>
         </is>
       </c>
     </row>
@@ -31416,7 +31416,7 @@
       <c r="AD364" s="2" t="inlineStr"/>
       <c r="AE364" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01899; NV lic #B01293</t>
+          <t>NV lic #B01899</t>
         </is>
       </c>
     </row>
@@ -31501,7 +31501,7 @@
       <c r="AD365" s="2" t="inlineStr"/>
       <c r="AE365" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01302; NV lic #B01661</t>
+          <t>NV lic #B01302</t>
         </is>
       </c>
     </row>
@@ -31926,7 +31926,7 @@
       <c r="AD370" s="2" t="inlineStr"/>
       <c r="AE370" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00531; disciplinary action on record</t>
+          <t>NV lic #B00531</t>
         </is>
       </c>
     </row>
@@ -32347,7 +32347,7 @@
       <c r="AD375" s="2" t="inlineStr"/>
       <c r="AE375" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01207; disciplinary action on record</t>
+          <t>NV lic #B01207</t>
         </is>
       </c>
     </row>
@@ -32432,7 +32432,7 @@
       <c r="AD376" s="2" t="inlineStr"/>
       <c r="AE376" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00825; NV lic #B00270</t>
+          <t>NV lic #B00825</t>
         </is>
       </c>
     </row>
@@ -33792,7 +33792,7 @@
       <c r="AD392" s="2" t="inlineStr"/>
       <c r="AE392" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01097; disciplinary action on record</t>
+          <t>NV lic #B01097</t>
         </is>
       </c>
     </row>
@@ -33877,7 +33877,7 @@
       <c r="AD393" s="2" t="inlineStr"/>
       <c r="AE393" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01098; disciplinary action on record</t>
+          <t>NV lic #B01098</t>
         </is>
       </c>
     </row>
@@ -34727,7 +34727,7 @@
       <c r="AD403" s="2" t="inlineStr"/>
       <c r="AE403" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01349; disciplinary action on record</t>
+          <t>NV lic #B01349</t>
         </is>
       </c>
     </row>
@@ -36407,7 +36407,7 @@
       <c r="AD423" s="2" t="inlineStr"/>
       <c r="AE423" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01023; disciplinary action on record</t>
+          <t>NV lic #B01023</t>
         </is>
       </c>
     </row>
@@ -37642,7 +37642,7 @@
       <c r="AD438" s="2" t="inlineStr"/>
       <c r="AE438" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01356; disciplinary action on record</t>
+          <t>NV lic #B01356</t>
         </is>
       </c>
     </row>
@@ -38735,7 +38735,7 @@
       <c r="AD451" s="2" t="inlineStr"/>
       <c r="AE451" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01502; NV lic #B01714</t>
+          <t>NV lic #B01502</t>
         </is>
       </c>
     </row>
@@ -39654,7 +39654,7 @@
       <c r="AD462" s="2" t="inlineStr"/>
       <c r="AE462" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01548; NV lic #B00827</t>
+          <t>NV lic #B01548</t>
         </is>
       </c>
     </row>
@@ -40241,7 +40241,7 @@
       <c r="AD469" s="2" t="inlineStr"/>
       <c r="AE469" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00757; NV lic #B01867</t>
+          <t>NV lic #B00757</t>
         </is>
       </c>
     </row>
@@ -40411,7 +40411,7 @@
       <c r="AD471" s="2" t="inlineStr"/>
       <c r="AE471" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00567; disciplinary action on record; NV lic #B0998</t>
+          <t>NV lic #B00567</t>
         </is>
       </c>
     </row>
@@ -41006,7 +41006,7 @@
       <c r="AD478" s="2" t="inlineStr"/>
       <c r="AE478" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01391; disciplinary action on record</t>
+          <t>NV lic #B01391</t>
         </is>
       </c>
     </row>
@@ -42107,7 +42107,7 @@
       <c r="AD491" s="2" t="inlineStr"/>
       <c r="AE491" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00308; NV lic #B00373</t>
+          <t>NV lic #B00308</t>
         </is>
       </c>
     </row>
@@ -42447,7 +42447,7 @@
       <c r="AD495" s="2" t="inlineStr"/>
       <c r="AE495" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02080; NV lic #B00808</t>
+          <t>NV lic #B02080</t>
         </is>
       </c>
     </row>
@@ -42702,7 +42702,7 @@
       <c r="AD498" s="2" t="inlineStr"/>
       <c r="AE498" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01973; NV lic #B00679</t>
+          <t>NV lic #B01973</t>
         </is>
       </c>
     </row>
@@ -43807,7 +43807,7 @@
       <c r="AD511" s="2" t="inlineStr"/>
       <c r="AE511" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01437; NV lic #B00190</t>
+          <t>NV lic #B01437</t>
         </is>
       </c>
     </row>
@@ -45932,7 +45932,7 @@
       <c r="AD536" s="2" t="inlineStr"/>
       <c r="AE536" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00525; disciplinary action on record</t>
+          <t>NV lic #B00525</t>
         </is>
       </c>
     </row>
@@ -46187,7 +46187,7 @@
       <c r="AD539" s="2" t="inlineStr"/>
       <c r="AE539" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00668; disciplinary action on record</t>
+          <t>NV lic #B00668</t>
         </is>
       </c>
     </row>
@@ -46782,7 +46782,7 @@
       <c r="AD546" s="2" t="inlineStr"/>
       <c r="AE546" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00200; disciplinary action on record</t>
+          <t>NV lic #B00200</t>
         </is>
       </c>
     </row>
@@ -47207,7 +47207,7 @@
       <c r="AD551" s="2" t="inlineStr"/>
       <c r="AE551" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00705; disciplinary action on record; NV lic #B00293</t>
+          <t>NV lic #B00705</t>
         </is>
       </c>
     </row>
@@ -47377,7 +47377,7 @@
       <c r="AD553" s="2" t="inlineStr"/>
       <c r="AE553" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01862; NV lic #B01899</t>
+          <t>NV lic #B01862</t>
         </is>
       </c>
     </row>
@@ -47632,7 +47632,7 @@
       <c r="AD556" s="2" t="inlineStr"/>
       <c r="AE556" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00294; disciplinary action on record</t>
+          <t>NV lic #B00294</t>
         </is>
       </c>
     </row>
@@ -47717,7 +47717,7 @@
       <c r="AD557" s="2" t="inlineStr"/>
       <c r="AE557" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01545; disciplinary action on record</t>
+          <t>NV lic #B01545</t>
         </is>
       </c>
     </row>
@@ -48300,7 +48300,7 @@
       <c r="AD564" s="2" t="inlineStr"/>
       <c r="AE564" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00962; disciplinary action on record</t>
+          <t>NV lic #B00962</t>
         </is>
       </c>
     </row>
@@ -48624,7 +48624,7 @@
       <c r="AD568" s="2" t="inlineStr"/>
       <c r="AE568" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00334; disciplinary action on record</t>
+          <t>NV lic #B00334</t>
         </is>
       </c>
     </row>
@@ -48786,7 +48786,7 @@
       <c r="AD570" s="2" t="inlineStr"/>
       <c r="AE570" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00262; disciplinary action on record</t>
+          <t>NV lic #B00262</t>
         </is>
       </c>
     </row>
@@ -49596,7 +49596,7 @@
       <c r="AD580" s="2" t="inlineStr"/>
       <c r="AE580" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01008; disciplinary action on record</t>
+          <t>NV lic #B01008</t>
         </is>
       </c>
     </row>
@@ -49758,7 +49758,7 @@
       <c r="AD582" s="2" t="inlineStr"/>
       <c r="AE582" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01082; disciplinary action on record</t>
+          <t>NV lic #B01082</t>
         </is>
       </c>
     </row>
@@ -49831,7 +49831,7 @@
       <c r="AD583" s="2" t="inlineStr"/>
       <c r="AE583" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01508; no individual NPI â find clinic to enrich; disciplinary action on record</t>
+          <t>NV lic #B01508</t>
         </is>
       </c>
     </row>
@@ -49904,7 +49904,7 @@
       <c r="AD584" s="2" t="inlineStr"/>
       <c r="AE584" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00284; no individual NPI â find clinic to enrich; disciplinary action on record</t>
+          <t>NV lic #B00284</t>
         </is>
       </c>
     </row>
@@ -49977,7 +49977,7 @@
       <c r="AD585" s="2" t="inlineStr"/>
       <c r="AE585" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01516; no individual NPI â find clinic to enrich; disciplinary action on record</t>
+          <t>NV lic #B01516</t>
         </is>
       </c>
     </row>
@@ -50050,7 +50050,7 @@
       <c r="AD586" s="2" t="inlineStr"/>
       <c r="AE586" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00888; no individual NPI â find clinic to enrich; disciplinary action on record</t>
+          <t>NV lic #B00888</t>
         </is>
       </c>
     </row>
@@ -50119,7 +50119,7 @@
       <c r="AD587" s="2" t="inlineStr"/>
       <c r="AE587" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00678; no individual NPI â find clinic to enrich; disciplinary action on record</t>
+          <t>NV lic #B00678</t>
         </is>
       </c>
     </row>
@@ -50192,7 +50192,7 @@
       <c r="AD588" s="2" t="inlineStr"/>
       <c r="AE588" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00449; no individual NPI â find clinic to enrich; disciplinary action on record</t>
+          <t>NV lic #B00449</t>
         </is>
       </c>
     </row>
@@ -50265,7 +50265,7 @@
       <c r="AD589" s="2" t="inlineStr"/>
       <c r="AE589" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00309; no individual NPI â find clinic to enrich; disciplinary action on record</t>
+          <t>NV lic #B00309</t>
         </is>
       </c>
     </row>
@@ -50338,7 +50338,7 @@
       <c r="AD590" s="2" t="inlineStr"/>
       <c r="AE590" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01883; no individual NPI â find clinic to enrich; disciplinary action on record</t>
+          <t>NV lic #B01883</t>
         </is>
       </c>
     </row>
@@ -50411,7 +50411,7 @@
       <c r="AD591" s="2" t="inlineStr"/>
       <c r="AE591" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00382; no individual NPI â find clinic to enrich; disciplinary action on record</t>
+          <t>NV lic #B00382</t>
         </is>
       </c>
     </row>
@@ -50484,7 +50484,7 @@
       <c r="AD592" s="2" t="inlineStr"/>
       <c r="AE592" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01618; no individual NPI â find clinic to enrich; disciplinary action on record</t>
+          <t>NV lic #B01618</t>
         </is>
       </c>
     </row>
@@ -50557,7 +50557,7 @@
       <c r="AD593" s="2" t="inlineStr"/>
       <c r="AE593" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01519; no individual NPI â find clinic to enrich; disciplinary action on record</t>
+          <t>NV lic #B01519</t>
         </is>
       </c>
     </row>
@@ -50630,7 +50630,7 @@
       <c r="AD594" s="2" t="inlineStr"/>
       <c r="AE594" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00747; no individual NPI â find clinic to enrich; disciplinary action on record</t>
+          <t>NV lic #B00747</t>
         </is>
       </c>
     </row>
@@ -50703,7 +50703,7 @@
       <c r="AD595" s="2" t="inlineStr"/>
       <c r="AE595" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01801; no individual NPI â find clinic to enrich; disciplinary action on record</t>
+          <t>NV lic #B01801</t>
         </is>
       </c>
     </row>
@@ -50776,7 +50776,7 @@
       <c r="AD596" s="2" t="inlineStr"/>
       <c r="AE596" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00527; no individual NPI â find clinic to enrich; disciplinary action on record</t>
+          <t>NV lic #B00527</t>
         </is>
       </c>
     </row>
@@ -50849,7 +50849,7 @@
       <c r="AD597" s="2" t="inlineStr"/>
       <c r="AE597" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01800; no individual NPI â find clinic to enrich; disciplinary action on record</t>
+          <t>NV lic #B01800</t>
         </is>
       </c>
     </row>
@@ -50922,7 +50922,7 @@
       <c r="AD598" s="2" t="inlineStr"/>
       <c r="AE598" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01781; no individual NPI â find clinic to enrich; disciplinary action on record</t>
+          <t>NV lic #B01781</t>
         </is>
       </c>
     </row>
@@ -50995,7 +50995,7 @@
       <c r="AD599" s="2" t="inlineStr"/>
       <c r="AE599" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01636; no individual NPI â find clinic to enrich; disciplinary action on record</t>
+          <t>NV lic #B01636</t>
         </is>
       </c>
     </row>
@@ -51068,7 +51068,7 @@
       <c r="AD600" s="2" t="inlineStr"/>
       <c r="AE600" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01079; no individual NPI â find clinic to enrich; disciplinary action on record</t>
+          <t>NV lic #B01079</t>
         </is>
       </c>
     </row>
@@ -51141,7 +51141,7 @@
       <c r="AD601" s="2" t="inlineStr"/>
       <c r="AE601" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01038; no individual NPI â find clinic to enrich; disciplinary action on record</t>
+          <t>NV lic #B01038</t>
         </is>
       </c>
     </row>
@@ -51214,7 +51214,7 @@
       <c r="AD602" s="2" t="inlineStr"/>
       <c r="AE602" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01818; no individual NPI â find clinic to enrich; disciplinary action on record</t>
+          <t>NV lic #B01818</t>
         </is>
       </c>
     </row>
@@ -51287,7 +51287,7 @@
       <c r="AD603" s="2" t="inlineStr"/>
       <c r="AE603" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00872; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00872</t>
         </is>
       </c>
     </row>
@@ -51360,7 +51360,7 @@
       <c r="AD604" s="2" t="inlineStr"/>
       <c r="AE604" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01815; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01815</t>
         </is>
       </c>
     </row>
@@ -51433,7 +51433,7 @@
       <c r="AD605" s="2" t="inlineStr"/>
       <c r="AE605" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02095; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02095</t>
         </is>
       </c>
     </row>
@@ -51506,7 +51506,7 @@
       <c r="AD606" s="2" t="inlineStr"/>
       <c r="AE606" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01339; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01339</t>
         </is>
       </c>
     </row>
@@ -51579,7 +51579,7 @@
       <c r="AD607" s="2" t="inlineStr"/>
       <c r="AE607" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00866; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00866</t>
         </is>
       </c>
     </row>
@@ -51652,7 +51652,7 @@
       <c r="AD608" s="2" t="inlineStr"/>
       <c r="AE608" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01923; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01923</t>
         </is>
       </c>
     </row>
@@ -51725,7 +51725,7 @@
       <c r="AD609" s="2" t="inlineStr"/>
       <c r="AE609" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01787; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01787</t>
         </is>
       </c>
     </row>
@@ -51798,7 +51798,7 @@
       <c r="AD610" s="2" t="inlineStr"/>
       <c r="AE610" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02070; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02070</t>
         </is>
       </c>
     </row>
@@ -51871,7 +51871,7 @@
       <c r="AD611" s="2" t="inlineStr"/>
       <c r="AE611" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02052; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02052</t>
         </is>
       </c>
     </row>
@@ -51944,7 +51944,7 @@
       <c r="AD612" s="2" t="inlineStr"/>
       <c r="AE612" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01993; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01993</t>
         </is>
       </c>
     </row>
@@ -52013,7 +52013,7 @@
       <c r="AD613" s="2" t="inlineStr"/>
       <c r="AE613" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01847; no individual NPI â find clinic to enrich; NV lic #B01425</t>
+          <t>NV lic #B01847</t>
         </is>
       </c>
     </row>
@@ -52086,7 +52086,7 @@
       <c r="AD614" s="2" t="inlineStr"/>
       <c r="AE614" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00862; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00862</t>
         </is>
       </c>
     </row>
@@ -52159,7 +52159,7 @@
       <c r="AD615" s="2" t="inlineStr"/>
       <c r="AE615" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00959; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00959</t>
         </is>
       </c>
     </row>
@@ -52232,7 +52232,7 @@
       <c r="AD616" s="2" t="inlineStr"/>
       <c r="AE616" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01573; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01573</t>
         </is>
       </c>
     </row>
@@ -52305,7 +52305,7 @@
       <c r="AD617" s="2" t="inlineStr"/>
       <c r="AE617" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01641; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01641</t>
         </is>
       </c>
     </row>
@@ -52378,7 +52378,7 @@
       <c r="AD618" s="2" t="inlineStr"/>
       <c r="AE618" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00960; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00960</t>
         </is>
       </c>
     </row>
@@ -52451,7 +52451,7 @@
       <c r="AD619" s="2" t="inlineStr"/>
       <c r="AE619" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02155; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02155</t>
         </is>
       </c>
     </row>
@@ -52524,7 +52524,7 @@
       <c r="AD620" s="2" t="inlineStr"/>
       <c r="AE620" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02156; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02156</t>
         </is>
       </c>
     </row>
@@ -52597,7 +52597,7 @@
       <c r="AD621" s="2" t="inlineStr"/>
       <c r="AE621" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01712; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01712</t>
         </is>
       </c>
     </row>
@@ -52670,7 +52670,7 @@
       <c r="AD622" s="2" t="inlineStr"/>
       <c r="AE622" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02028; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02028</t>
         </is>
       </c>
     </row>
@@ -52743,7 +52743,7 @@
       <c r="AD623" s="2" t="inlineStr"/>
       <c r="AE623" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00672; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00672</t>
         </is>
       </c>
     </row>
@@ -52816,7 +52816,7 @@
       <c r="AD624" s="2" t="inlineStr"/>
       <c r="AE624" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01210; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01210</t>
         </is>
       </c>
     </row>
@@ -52885,7 +52885,7 @@
       <c r="AD625" s="2" t="inlineStr"/>
       <c r="AE625" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01350; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01350</t>
         </is>
       </c>
     </row>
@@ -52958,7 +52958,7 @@
       <c r="AD626" s="2" t="inlineStr"/>
       <c r="AE626" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02141; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02141</t>
         </is>
       </c>
     </row>
@@ -53031,7 +53031,7 @@
       <c r="AD627" s="2" t="inlineStr"/>
       <c r="AE627" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01319; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01319</t>
         </is>
       </c>
     </row>
@@ -53104,7 +53104,7 @@
       <c r="AD628" s="2" t="inlineStr"/>
       <c r="AE628" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02154; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02154</t>
         </is>
       </c>
     </row>
@@ -53173,7 +53173,7 @@
       <c r="AD629" s="2" t="inlineStr"/>
       <c r="AE629" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00492; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00492</t>
         </is>
       </c>
     </row>
@@ -53242,7 +53242,7 @@
       <c r="AD630" s="2" t="inlineStr"/>
       <c r="AE630" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01917; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01917</t>
         </is>
       </c>
     </row>
@@ -53311,7 +53311,7 @@
       <c r="AD631" s="2" t="inlineStr"/>
       <c r="AE631" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02062; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02062</t>
         </is>
       </c>
     </row>
@@ -53384,7 +53384,7 @@
       <c r="AD632" s="2" t="inlineStr"/>
       <c r="AE632" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01740; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01740</t>
         </is>
       </c>
     </row>
@@ -53457,7 +53457,7 @@
       <c r="AD633" s="2" t="inlineStr"/>
       <c r="AE633" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01840; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01840</t>
         </is>
       </c>
     </row>
@@ -53526,7 +53526,7 @@
       <c r="AD634" s="2" t="inlineStr"/>
       <c r="AE634" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00357; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00357</t>
         </is>
       </c>
     </row>
@@ -53599,7 +53599,7 @@
       <c r="AD635" s="2" t="inlineStr"/>
       <c r="AE635" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01639; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01639</t>
         </is>
       </c>
     </row>
@@ -53672,7 +53672,7 @@
       <c r="AD636" s="2" t="inlineStr"/>
       <c r="AE636" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01612; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01612</t>
         </is>
       </c>
     </row>
@@ -53745,7 +53745,7 @@
       <c r="AD637" s="2" t="inlineStr"/>
       <c r="AE637" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02101; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02101</t>
         </is>
       </c>
     </row>
@@ -53814,7 +53814,7 @@
       <c r="AD638" s="2" t="inlineStr"/>
       <c r="AE638" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01477; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01477</t>
         </is>
       </c>
     </row>
@@ -53887,7 +53887,7 @@
       <c r="AD639" s="2" t="inlineStr"/>
       <c r="AE639" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02124; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02124</t>
         </is>
       </c>
     </row>
@@ -53956,7 +53956,7 @@
       <c r="AD640" s="2" t="inlineStr"/>
       <c r="AE640" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00096; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00096</t>
         </is>
       </c>
     </row>
@@ -54029,7 +54029,7 @@
       <c r="AD641" s="2" t="inlineStr"/>
       <c r="AE641" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01889; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01889</t>
         </is>
       </c>
     </row>
@@ -54102,7 +54102,7 @@
       <c r="AD642" s="2" t="inlineStr"/>
       <c r="AE642" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02103; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02103</t>
         </is>
       </c>
     </row>
@@ -54175,7 +54175,7 @@
       <c r="AD643" s="2" t="inlineStr"/>
       <c r="AE643" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02123; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02123</t>
         </is>
       </c>
     </row>
@@ -54248,7 +54248,7 @@
       <c r="AD644" s="2" t="inlineStr"/>
       <c r="AE644" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01320; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01320</t>
         </is>
       </c>
     </row>
@@ -54317,7 +54317,7 @@
       <c r="AD645" s="2" t="inlineStr"/>
       <c r="AE645" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01819; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01819</t>
         </is>
       </c>
     </row>
@@ -54390,7 +54390,7 @@
       <c r="AD646" s="2" t="inlineStr"/>
       <c r="AE646" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01965; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01965</t>
         </is>
       </c>
     </row>
@@ -54463,7 +54463,7 @@
       <c r="AD647" s="2" t="inlineStr"/>
       <c r="AE647" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01352; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01352</t>
         </is>
       </c>
     </row>
@@ -54536,7 +54536,7 @@
       <c r="AD648" s="2" t="inlineStr"/>
       <c r="AE648" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01834; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01834</t>
         </is>
       </c>
     </row>
@@ -54609,7 +54609,7 @@
       <c r="AD649" s="2" t="inlineStr"/>
       <c r="AE649" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01395; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01395</t>
         </is>
       </c>
     </row>
@@ -54682,7 +54682,7 @@
       <c r="AD650" s="2" t="inlineStr"/>
       <c r="AE650" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01977; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01977</t>
         </is>
       </c>
     </row>
@@ -54755,7 +54755,7 @@
       <c r="AD651" s="2" t="inlineStr"/>
       <c r="AE651" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00694; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00694</t>
         </is>
       </c>
     </row>
@@ -54828,7 +54828,7 @@
       <c r="AD652" s="2" t="inlineStr"/>
       <c r="AE652" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02133; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02133</t>
         </is>
       </c>
     </row>
@@ -54901,7 +54901,7 @@
       <c r="AD653" s="2" t="inlineStr"/>
       <c r="AE653" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02104; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02104</t>
         </is>
       </c>
     </row>
@@ -54974,7 +54974,7 @@
       <c r="AD654" s="2" t="inlineStr"/>
       <c r="AE654" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01654; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01654</t>
         </is>
       </c>
     </row>
@@ -55043,7 +55043,7 @@
       <c r="AD655" s="2" t="inlineStr"/>
       <c r="AE655" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02098; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02098</t>
         </is>
       </c>
     </row>
@@ -55116,7 +55116,7 @@
       <c r="AD656" s="2" t="inlineStr"/>
       <c r="AE656" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01758; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01758</t>
         </is>
       </c>
     </row>
@@ -55189,7 +55189,7 @@
       <c r="AD657" s="2" t="inlineStr"/>
       <c r="AE657" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01253; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01253</t>
         </is>
       </c>
     </row>
@@ -55262,7 +55262,7 @@
       <c r="AD658" s="2" t="inlineStr"/>
       <c r="AE658" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01586; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01586</t>
         </is>
       </c>
     </row>
@@ -55335,7 +55335,7 @@
       <c r="AD659" s="2" t="inlineStr"/>
       <c r="AE659" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02077; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02077</t>
         </is>
       </c>
     </row>
@@ -55408,7 +55408,7 @@
       <c r="AD660" s="2" t="inlineStr"/>
       <c r="AE660" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00806; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00806</t>
         </is>
       </c>
     </row>
@@ -55481,7 +55481,7 @@
       <c r="AD661" s="2" t="inlineStr"/>
       <c r="AE661" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02144; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02144</t>
         </is>
       </c>
     </row>
@@ -55550,7 +55550,7 @@
       <c r="AD662" s="2" t="inlineStr"/>
       <c r="AE662" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00142; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00142</t>
         </is>
       </c>
     </row>
@@ -55623,7 +55623,7 @@
       <c r="AD663" s="2" t="inlineStr"/>
       <c r="AE663" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00963; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00963</t>
         </is>
       </c>
     </row>
@@ -55696,7 +55696,7 @@
       <c r="AD664" s="2" t="inlineStr"/>
       <c r="AE664" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02063; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02063</t>
         </is>
       </c>
     </row>
@@ -55769,7 +55769,7 @@
       <c r="AD665" s="2" t="inlineStr"/>
       <c r="AE665" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02087; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02087</t>
         </is>
       </c>
     </row>
@@ -55842,7 +55842,7 @@
       <c r="AD666" s="2" t="inlineStr"/>
       <c r="AE666" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01790; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01790</t>
         </is>
       </c>
     </row>
@@ -55915,7 +55915,7 @@
       <c r="AD667" s="2" t="inlineStr"/>
       <c r="AE667" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02066; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02066</t>
         </is>
       </c>
     </row>
@@ -55988,7 +55988,7 @@
       <c r="AD668" s="2" t="inlineStr"/>
       <c r="AE668" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01986; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01986</t>
         </is>
       </c>
     </row>
@@ -56061,7 +56061,7 @@
       <c r="AD669" s="2" t="inlineStr"/>
       <c r="AE669" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00829; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00829</t>
         </is>
       </c>
     </row>
@@ -56134,7 +56134,7 @@
       <c r="AD670" s="2" t="inlineStr"/>
       <c r="AE670" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02096; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02096</t>
         </is>
       </c>
     </row>
@@ -56203,7 +56203,7 @@
       <c r="AD671" s="2" t="inlineStr"/>
       <c r="AE671" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01454; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01454</t>
         </is>
       </c>
     </row>
@@ -56276,7 +56276,7 @@
       <c r="AD672" s="2" t="inlineStr"/>
       <c r="AE672" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01768; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01768</t>
         </is>
       </c>
     </row>
@@ -56349,7 +56349,7 @@
       <c r="AD673" s="2" t="inlineStr"/>
       <c r="AE673" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01311; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01311</t>
         </is>
       </c>
     </row>
@@ -56422,7 +56422,7 @@
       <c r="AD674" s="2" t="inlineStr"/>
       <c r="AE674" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02075; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02075</t>
         </is>
       </c>
     </row>
@@ -56495,7 +56495,7 @@
       <c r="AD675" s="2" t="inlineStr"/>
       <c r="AE675" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01972; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01972</t>
         </is>
       </c>
     </row>
@@ -56568,7 +56568,7 @@
       <c r="AD676" s="2" t="inlineStr"/>
       <c r="AE676" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01014; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01014</t>
         </is>
       </c>
     </row>
@@ -56641,7 +56641,7 @@
       <c r="AD677" s="2" t="inlineStr"/>
       <c r="AE677" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01813; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01813</t>
         </is>
       </c>
     </row>
@@ -56714,7 +56714,7 @@
       <c r="AD678" s="2" t="inlineStr"/>
       <c r="AE678" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02072; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02072</t>
         </is>
       </c>
     </row>
@@ -56787,7 +56787,7 @@
       <c r="AD679" s="2" t="inlineStr"/>
       <c r="AE679" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01531; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01531</t>
         </is>
       </c>
     </row>
@@ -56856,7 +56856,7 @@
       <c r="AD680" s="2" t="inlineStr"/>
       <c r="AE680" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01896; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01896</t>
         </is>
       </c>
     </row>
@@ -56929,7 +56929,7 @@
       <c r="AD681" s="2" t="inlineStr"/>
       <c r="AE681" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00276; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00276</t>
         </is>
       </c>
     </row>
@@ -56998,7 +56998,7 @@
       <c r="AD682" s="2" t="inlineStr"/>
       <c r="AE682" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00925; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00925</t>
         </is>
       </c>
     </row>
@@ -57071,7 +57071,7 @@
       <c r="AD683" s="2" t="inlineStr"/>
       <c r="AE683" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02138; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02138</t>
         </is>
       </c>
     </row>
@@ -57144,7 +57144,7 @@
       <c r="AD684" s="2" t="inlineStr"/>
       <c r="AE684" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02064; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02064</t>
         </is>
       </c>
     </row>
@@ -57217,7 +57217,7 @@
       <c r="AD685" s="2" t="inlineStr"/>
       <c r="AE685" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01999; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01999</t>
         </is>
       </c>
     </row>
@@ -57286,7 +57286,7 @@
       <c r="AD686" s="2" t="inlineStr"/>
       <c r="AE686" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02065; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02065</t>
         </is>
       </c>
     </row>
@@ -57359,7 +57359,7 @@
       <c r="AD687" s="2" t="inlineStr"/>
       <c r="AE687" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02145; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02145</t>
         </is>
       </c>
     </row>
@@ -57432,7 +57432,7 @@
       <c r="AD688" s="2" t="inlineStr"/>
       <c r="AE688" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01950; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01950</t>
         </is>
       </c>
     </row>
@@ -57505,7 +57505,7 @@
       <c r="AD689" s="2" t="inlineStr"/>
       <c r="AE689" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02162; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02162</t>
         </is>
       </c>
     </row>
@@ -57578,7 +57578,7 @@
       <c r="AD690" s="2" t="inlineStr"/>
       <c r="AE690" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01911; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01911</t>
         </is>
       </c>
     </row>
@@ -57651,7 +57651,7 @@
       <c r="AD691" s="2" t="inlineStr"/>
       <c r="AE691" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02116; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02116</t>
         </is>
       </c>
     </row>
@@ -57724,7 +57724,7 @@
       <c r="AD692" s="2" t="inlineStr"/>
       <c r="AE692" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01968; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01968</t>
         </is>
       </c>
     </row>
@@ -57797,7 +57797,7 @@
       <c r="AD693" s="2" t="inlineStr"/>
       <c r="AE693" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01167; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01167</t>
         </is>
       </c>
     </row>
@@ -57870,7 +57870,7 @@
       <c r="AD694" s="2" t="inlineStr"/>
       <c r="AE694" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01811; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01811</t>
         </is>
       </c>
     </row>
@@ -57939,7 +57939,7 @@
       <c r="AD695" s="2" t="inlineStr"/>
       <c r="AE695" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02102; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02102</t>
         </is>
       </c>
     </row>
@@ -58008,7 +58008,7 @@
       <c r="AD696" s="2" t="inlineStr"/>
       <c r="AE696" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02135; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02135</t>
         </is>
       </c>
     </row>
@@ -58081,7 +58081,7 @@
       <c r="AD697" s="2" t="inlineStr"/>
       <c r="AE697" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01298; no individual NPI â find clinic to enrich; NV lic #B00221</t>
+          <t>NV lic #B01298</t>
         </is>
       </c>
     </row>
@@ -58154,7 +58154,7 @@
       <c r="AD698" s="2" t="inlineStr"/>
       <c r="AE698" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01989; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01989</t>
         </is>
       </c>
     </row>
@@ -58227,7 +58227,7 @@
       <c r="AD699" s="2" t="inlineStr"/>
       <c r="AE699" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02109; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02109</t>
         </is>
       </c>
     </row>
@@ -58300,7 +58300,7 @@
       <c r="AD700" s="2" t="inlineStr"/>
       <c r="AE700" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01325; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01325</t>
         </is>
       </c>
     </row>
@@ -58369,7 +58369,7 @@
       <c r="AD701" s="2" t="inlineStr"/>
       <c r="AE701" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02134; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02134</t>
         </is>
       </c>
     </row>
@@ -58442,7 +58442,7 @@
       <c r="AD702" s="2" t="inlineStr"/>
       <c r="AE702" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02059; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02059</t>
         </is>
       </c>
     </row>
@@ -58511,7 +58511,7 @@
       <c r="AD703" s="2" t="inlineStr"/>
       <c r="AE703" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01814; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01814</t>
         </is>
       </c>
     </row>
@@ -58584,7 +58584,7 @@
       <c r="AD704" s="2" t="inlineStr"/>
       <c r="AE704" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01809; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01809</t>
         </is>
       </c>
     </row>
@@ -58657,7 +58657,7 @@
       <c r="AD705" s="2" t="inlineStr"/>
       <c r="AE705" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02042; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02042</t>
         </is>
       </c>
     </row>
@@ -58730,7 +58730,7 @@
       <c r="AD706" s="2" t="inlineStr"/>
       <c r="AE706" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02083; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02083</t>
         </is>
       </c>
     </row>
@@ -58803,7 +58803,7 @@
       <c r="AD707" s="2" t="inlineStr"/>
       <c r="AE707" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02106; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02106</t>
         </is>
       </c>
     </row>
@@ -58876,7 +58876,7 @@
       <c r="AD708" s="2" t="inlineStr"/>
       <c r="AE708" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01777; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01777</t>
         </is>
       </c>
     </row>
@@ -58949,7 +58949,7 @@
       <c r="AD709" s="2" t="inlineStr"/>
       <c r="AE709" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01953; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01953</t>
         </is>
       </c>
     </row>
@@ -59018,7 +59018,7 @@
       <c r="AD710" s="2" t="inlineStr"/>
       <c r="AE710" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00470; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00470</t>
         </is>
       </c>
     </row>
@@ -59091,7 +59091,7 @@
       <c r="AD711" s="2" t="inlineStr"/>
       <c r="AE711" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02114; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02114</t>
         </is>
       </c>
     </row>
@@ -59164,7 +59164,7 @@
       <c r="AD712" s="2" t="inlineStr"/>
       <c r="AE712" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01920; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01920</t>
         </is>
       </c>
     </row>
@@ -59237,7 +59237,7 @@
       <c r="AD713" s="2" t="inlineStr"/>
       <c r="AE713" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02165; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02165</t>
         </is>
       </c>
     </row>
@@ -59310,7 +59310,7 @@
       <c r="AD714" s="2" t="inlineStr"/>
       <c r="AE714" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02017; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02017</t>
         </is>
       </c>
     </row>
@@ -59383,7 +59383,7 @@
       <c r="AD715" s="2" t="inlineStr"/>
       <c r="AE715" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02054; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02054</t>
         </is>
       </c>
     </row>
@@ -59456,7 +59456,7 @@
       <c r="AD716" s="2" t="inlineStr"/>
       <c r="AE716" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01970; no individual NPI â find clinic to enrich; NV lic #B00594</t>
+          <t>NV lic #B01970</t>
         </is>
       </c>
     </row>
@@ -59529,7 +59529,7 @@
       <c r="AD717" s="2" t="inlineStr"/>
       <c r="AE717" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01396; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01396</t>
         </is>
       </c>
     </row>
@@ -59602,7 +59602,7 @@
       <c r="AD718" s="2" t="inlineStr"/>
       <c r="AE718" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01368; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01368</t>
         </is>
       </c>
     </row>
@@ -59675,7 +59675,7 @@
       <c r="AD719" s="2" t="inlineStr"/>
       <c r="AE719" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00769; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00769</t>
         </is>
       </c>
     </row>
@@ -59748,7 +59748,7 @@
       <c r="AD720" s="2" t="inlineStr"/>
       <c r="AE720" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02120; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02120</t>
         </is>
       </c>
     </row>
@@ -59821,7 +59821,7 @@
       <c r="AD721" s="2" t="inlineStr"/>
       <c r="AE721" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01791; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01791</t>
         </is>
       </c>
     </row>
@@ -59890,7 +59890,7 @@
       <c r="AD722" s="2" t="inlineStr"/>
       <c r="AE722" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01947; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01947</t>
         </is>
       </c>
     </row>
@@ -59959,7 +59959,7 @@
       <c r="AD723" s="2" t="inlineStr"/>
       <c r="AE723" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01273; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01273</t>
         </is>
       </c>
     </row>
@@ -60032,7 +60032,7 @@
       <c r="AD724" s="2" t="inlineStr"/>
       <c r="AE724" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02079; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02079</t>
         </is>
       </c>
     </row>
@@ -60105,7 +60105,7 @@
       <c r="AD725" s="2" t="inlineStr"/>
       <c r="AE725" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02153; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02153</t>
         </is>
       </c>
     </row>
@@ -60178,7 +60178,7 @@
       <c r="AD726" s="2" t="inlineStr"/>
       <c r="AE726" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00843; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00843</t>
         </is>
       </c>
     </row>
@@ -60251,7 +60251,7 @@
       <c r="AD727" s="2" t="inlineStr"/>
       <c r="AE727" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01540; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01540</t>
         </is>
       </c>
     </row>
@@ -60324,7 +60324,7 @@
       <c r="AD728" s="2" t="inlineStr"/>
       <c r="AE728" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02113; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02113</t>
         </is>
       </c>
     </row>
@@ -60397,7 +60397,7 @@
       <c r="AD729" s="2" t="inlineStr"/>
       <c r="AE729" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02112; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02112</t>
         </is>
       </c>
     </row>
@@ -60470,7 +60470,7 @@
       <c r="AD730" s="2" t="inlineStr"/>
       <c r="AE730" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00742; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00742</t>
         </is>
       </c>
     </row>
@@ -60543,7 +60543,7 @@
       <c r="AD731" s="2" t="inlineStr"/>
       <c r="AE731" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01966; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01966</t>
         </is>
       </c>
     </row>
@@ -60616,7 +60616,7 @@
       <c r="AD732" s="2" t="inlineStr"/>
       <c r="AE732" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01590; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01590</t>
         </is>
       </c>
     </row>
@@ -60685,7 +60685,7 @@
       <c r="AD733" s="2" t="inlineStr"/>
       <c r="AE733" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02147; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02147</t>
         </is>
       </c>
     </row>
@@ -60758,7 +60758,7 @@
       <c r="AD734" s="2" t="inlineStr"/>
       <c r="AE734" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01901; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01901</t>
         </is>
       </c>
     </row>
@@ -60831,7 +60831,7 @@
       <c r="AD735" s="2" t="inlineStr"/>
       <c r="AE735" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00663; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00663</t>
         </is>
       </c>
     </row>
@@ -60900,7 +60900,7 @@
       <c r="AD736" s="2" t="inlineStr"/>
       <c r="AE736" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01846; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01846</t>
         </is>
       </c>
     </row>
@@ -60973,7 +60973,7 @@
       <c r="AD737" s="2" t="inlineStr"/>
       <c r="AE737" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01900; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01900</t>
         </is>
       </c>
     </row>
@@ -61046,7 +61046,7 @@
       <c r="AD738" s="2" t="inlineStr"/>
       <c r="AE738" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02161; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02161</t>
         </is>
       </c>
     </row>
@@ -61119,7 +61119,7 @@
       <c r="AD739" s="2" t="inlineStr"/>
       <c r="AE739" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02056; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02056</t>
         </is>
       </c>
     </row>
@@ -61192,7 +61192,7 @@
       <c r="AD740" s="2" t="inlineStr"/>
       <c r="AE740" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02086; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02086</t>
         </is>
       </c>
     </row>
@@ -61265,7 +61265,7 @@
       <c r="AD741" s="2" t="inlineStr"/>
       <c r="AE741" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02117; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02117</t>
         </is>
       </c>
     </row>
@@ -61334,7 +61334,7 @@
       <c r="AD742" s="2" t="inlineStr"/>
       <c r="AE742" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01940; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01940</t>
         </is>
       </c>
     </row>
@@ -61407,7 +61407,7 @@
       <c r="AD743" s="2" t="inlineStr"/>
       <c r="AE743" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02128; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02128</t>
         </is>
       </c>
     </row>
@@ -61476,7 +61476,7 @@
       <c r="AD744" s="2" t="inlineStr"/>
       <c r="AE744" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01943; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01943</t>
         </is>
       </c>
     </row>
@@ -61545,7 +61545,7 @@
       <c r="AD745" s="2" t="inlineStr"/>
       <c r="AE745" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01574; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01574</t>
         </is>
       </c>
     </row>
@@ -61618,7 +61618,7 @@
       <c r="AD746" s="2" t="inlineStr"/>
       <c r="AE746" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02130; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02130</t>
         </is>
       </c>
     </row>
@@ -61691,7 +61691,7 @@
       <c r="AD747" s="2" t="inlineStr"/>
       <c r="AE747" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02157; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02157</t>
         </is>
       </c>
     </row>
@@ -61764,7 +61764,7 @@
       <c r="AD748" s="2" t="inlineStr"/>
       <c r="AE748" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02159; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02159</t>
         </is>
       </c>
     </row>
@@ -61833,7 +61833,7 @@
       <c r="AD749" s="2" t="inlineStr"/>
       <c r="AE749" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02118; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02118</t>
         </is>
       </c>
     </row>
@@ -61906,7 +61906,7 @@
       <c r="AD750" s="2" t="inlineStr"/>
       <c r="AE750" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02076; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02076</t>
         </is>
       </c>
     </row>
@@ -61979,7 +61979,7 @@
       <c r="AD751" s="2" t="inlineStr"/>
       <c r="AE751" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02127; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02127</t>
         </is>
       </c>
     </row>
@@ -62052,7 +62052,7 @@
       <c r="AD752" s="2" t="inlineStr"/>
       <c r="AE752" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01382; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01382</t>
         </is>
       </c>
     </row>
@@ -62125,7 +62125,7 @@
       <c r="AD753" s="2" t="inlineStr"/>
       <c r="AE753" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01897; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01897</t>
         </is>
       </c>
     </row>
@@ -62194,7 +62194,7 @@
       <c r="AD754" s="2" t="inlineStr"/>
       <c r="AE754" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00618; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00618</t>
         </is>
       </c>
     </row>
@@ -62263,7 +62263,7 @@
       <c r="AD755" s="2" t="inlineStr"/>
       <c r="AE755" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02160; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02160</t>
         </is>
       </c>
     </row>
@@ -62336,7 +62336,7 @@
       <c r="AD756" s="2" t="inlineStr"/>
       <c r="AE756" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02057; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02057</t>
         </is>
       </c>
     </row>
@@ -62405,7 +62405,7 @@
       <c r="AD757" s="2" t="inlineStr"/>
       <c r="AE757" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01794; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01794</t>
         </is>
       </c>
     </row>
@@ -62474,7 +62474,7 @@
       <c r="AD758" s="2" t="inlineStr"/>
       <c r="AE758" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01854; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01854</t>
         </is>
       </c>
     </row>
@@ -62547,7 +62547,7 @@
       <c r="AD759" s="2" t="inlineStr"/>
       <c r="AE759" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01979; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01979</t>
         </is>
       </c>
     </row>
@@ -62616,7 +62616,7 @@
       <c r="AD760" s="2" t="inlineStr"/>
       <c r="AE760" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01865; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01865</t>
         </is>
       </c>
     </row>
@@ -62689,7 +62689,7 @@
       <c r="AD761" s="2" t="inlineStr"/>
       <c r="AE761" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01789; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01789</t>
         </is>
       </c>
     </row>
@@ -62762,7 +62762,7 @@
       <c r="AD762" s="2" t="inlineStr"/>
       <c r="AE762" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01932; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01932</t>
         </is>
       </c>
     </row>
@@ -62835,7 +62835,7 @@
       <c r="AD763" s="2" t="inlineStr"/>
       <c r="AE763" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01887; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01887</t>
         </is>
       </c>
     </row>
@@ -62908,7 +62908,7 @@
       <c r="AD764" s="2" t="inlineStr"/>
       <c r="AE764" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02050; no individual NPI â find clinic to enrich; NV lic #B00818</t>
+          <t>NV lic #B02050</t>
         </is>
       </c>
     </row>
@@ -62981,7 +62981,7 @@
       <c r="AD765" s="2" t="inlineStr"/>
       <c r="AE765" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01447; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01447</t>
         </is>
       </c>
     </row>
@@ -63050,7 +63050,7 @@
       <c r="AD766" s="2" t="inlineStr"/>
       <c r="AE766" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01092; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01092</t>
         </is>
       </c>
     </row>
@@ -63119,7 +63119,7 @@
       <c r="AD767" s="2" t="inlineStr"/>
       <c r="AE767" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01190; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01190</t>
         </is>
       </c>
     </row>
@@ -63192,7 +63192,7 @@
       <c r="AD768" s="2" t="inlineStr"/>
       <c r="AE768" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02048; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02048</t>
         </is>
       </c>
     </row>
@@ -63265,7 +63265,7 @@
       <c r="AD769" s="2" t="inlineStr"/>
       <c r="AE769" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00727; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00727</t>
         </is>
       </c>
     </row>
@@ -63338,7 +63338,7 @@
       <c r="AD770" s="2" t="inlineStr"/>
       <c r="AE770" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01091; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01091</t>
         </is>
       </c>
     </row>
@@ -63411,7 +63411,7 @@
       <c r="AD771" s="2" t="inlineStr"/>
       <c r="AE771" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01927; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01927</t>
         </is>
       </c>
     </row>
@@ -63484,7 +63484,7 @@
       <c r="AD772" s="2" t="inlineStr"/>
       <c r="AE772" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01442; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01442</t>
         </is>
       </c>
     </row>
@@ -63557,7 +63557,7 @@
       <c r="AD773" s="2" t="inlineStr"/>
       <c r="AE773" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01242; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01242</t>
         </is>
       </c>
     </row>
@@ -63630,7 +63630,7 @@
       <c r="AD774" s="2" t="inlineStr"/>
       <c r="AE774" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02163; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02163</t>
         </is>
       </c>
     </row>
@@ -63703,7 +63703,7 @@
       <c r="AD775" s="2" t="inlineStr"/>
       <c r="AE775" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02053; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02053</t>
         </is>
       </c>
     </row>
@@ -63776,7 +63776,7 @@
       <c r="AD776" s="2" t="inlineStr"/>
       <c r="AE776" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01982; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01982</t>
         </is>
       </c>
     </row>
@@ -63849,7 +63849,7 @@
       <c r="AD777" s="2" t="inlineStr"/>
       <c r="AE777" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01453; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01453</t>
         </is>
       </c>
     </row>
@@ -63922,7 +63922,7 @@
       <c r="AD778" s="2" t="inlineStr"/>
       <c r="AE778" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02019; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02019</t>
         </is>
       </c>
     </row>
@@ -63991,7 +63991,7 @@
       <c r="AD779" s="2" t="inlineStr"/>
       <c r="AE779" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01579; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01579</t>
         </is>
       </c>
     </row>
@@ -64064,7 +64064,7 @@
       <c r="AD780" s="2" t="inlineStr"/>
       <c r="AE780" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01904; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01904</t>
         </is>
       </c>
     </row>
@@ -64137,7 +64137,7 @@
       <c r="AD781" s="2" t="inlineStr"/>
       <c r="AE781" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01981; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01981</t>
         </is>
       </c>
     </row>
@@ -64206,7 +64206,7 @@
       <c r="AD782" s="2" t="inlineStr"/>
       <c r="AE782" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02093; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02093</t>
         </is>
       </c>
     </row>
@@ -64279,7 +64279,7 @@
       <c r="AD783" s="2" t="inlineStr"/>
       <c r="AE783" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01928; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01928</t>
         </is>
       </c>
     </row>
@@ -64348,7 +64348,7 @@
       <c r="AD784" s="2" t="inlineStr"/>
       <c r="AE784" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01853; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01853</t>
         </is>
       </c>
     </row>
@@ -64421,7 +64421,7 @@
       <c r="AD785" s="2" t="inlineStr"/>
       <c r="AE785" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00302; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00302</t>
         </is>
       </c>
     </row>
@@ -64494,7 +64494,7 @@
       <c r="AD786" s="2" t="inlineStr"/>
       <c r="AE786" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02024; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02024</t>
         </is>
       </c>
     </row>
@@ -64567,7 +64567,7 @@
       <c r="AD787" s="2" t="inlineStr"/>
       <c r="AE787" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01955; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01955</t>
         </is>
       </c>
     </row>
@@ -64640,7 +64640,7 @@
       <c r="AD788" s="2" t="inlineStr"/>
       <c r="AE788" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01888; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01888</t>
         </is>
       </c>
     </row>
@@ -64713,7 +64713,7 @@
       <c r="AD789" s="2" t="inlineStr"/>
       <c r="AE789" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B0992; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B0992</t>
         </is>
       </c>
     </row>
@@ -64786,7 +64786,7 @@
       <c r="AD790" s="2" t="inlineStr"/>
       <c r="AE790" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02151; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02151</t>
         </is>
       </c>
     </row>
@@ -64859,7 +64859,7 @@
       <c r="AD791" s="2" t="inlineStr"/>
       <c r="AE791" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02016; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02016</t>
         </is>
       </c>
     </row>
@@ -64932,7 +64932,7 @@
       <c r="AD792" s="2" t="inlineStr"/>
       <c r="AE792" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01225; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01225</t>
         </is>
       </c>
     </row>
@@ -65005,7 +65005,7 @@
       <c r="AD793" s="2" t="inlineStr"/>
       <c r="AE793" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01751; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01751</t>
         </is>
       </c>
     </row>
@@ -65078,7 +65078,7 @@
       <c r="AD794" s="2" t="inlineStr"/>
       <c r="AE794" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02146; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02146</t>
         </is>
       </c>
     </row>
@@ -65151,7 +65151,7 @@
       <c r="AD795" s="2" t="inlineStr"/>
       <c r="AE795" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00232; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00232</t>
         </is>
       </c>
     </row>
@@ -65224,7 +65224,7 @@
       <c r="AD796" s="2" t="inlineStr"/>
       <c r="AE796" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02045; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02045</t>
         </is>
       </c>
     </row>
@@ -65293,7 +65293,7 @@
       <c r="AD797" s="2" t="inlineStr"/>
       <c r="AE797" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02122; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02122</t>
         </is>
       </c>
     </row>
@@ -65366,7 +65366,7 @@
       <c r="AD798" s="2" t="inlineStr"/>
       <c r="AE798" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01582; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01582</t>
         </is>
       </c>
     </row>
@@ -65435,7 +65435,7 @@
       <c r="AD799" s="2" t="inlineStr"/>
       <c r="AE799" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02030; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02030</t>
         </is>
       </c>
     </row>
@@ -65508,7 +65508,7 @@
       <c r="AD800" s="2" t="inlineStr"/>
       <c r="AE800" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01980; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01980</t>
         </is>
       </c>
     </row>
@@ -65581,7 +65581,7 @@
       <c r="AD801" s="2" t="inlineStr"/>
       <c r="AE801" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01035; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01035</t>
         </is>
       </c>
     </row>
@@ -65650,7 +65650,7 @@
       <c r="AD802" s="2" t="inlineStr"/>
       <c r="AE802" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01583; no individual NPI â find clinic to enrich; NV lic #B00125</t>
+          <t>NV lic #B01583</t>
         </is>
       </c>
     </row>
@@ -65723,7 +65723,7 @@
       <c r="AD803" s="2" t="inlineStr"/>
       <c r="AE803" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00478; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00478</t>
         </is>
       </c>
     </row>
@@ -65796,7 +65796,7 @@
       <c r="AD804" s="2" t="inlineStr"/>
       <c r="AE804" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02029; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02029</t>
         </is>
       </c>
     </row>
@@ -65869,7 +65869,7 @@
       <c r="AD805" s="2" t="inlineStr"/>
       <c r="AE805" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01227; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01227</t>
         </is>
       </c>
     </row>
@@ -65942,7 +65942,7 @@
       <c r="AD806" s="2" t="inlineStr"/>
       <c r="AE806" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00317; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00317</t>
         </is>
       </c>
     </row>
@@ -66015,7 +66015,7 @@
       <c r="AD807" s="2" t="inlineStr"/>
       <c r="AE807" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02081; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02081</t>
         </is>
       </c>
     </row>
@@ -66084,7 +66084,7 @@
       <c r="AD808" s="2" t="inlineStr"/>
       <c r="AE808" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02049; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02049</t>
         </is>
       </c>
     </row>
@@ -66153,7 +66153,7 @@
       <c r="AD809" s="2" t="inlineStr"/>
       <c r="AE809" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01951; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01951</t>
         </is>
       </c>
     </row>
@@ -66226,7 +66226,7 @@
       <c r="AD810" s="2" t="inlineStr"/>
       <c r="AE810" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00292; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00292</t>
         </is>
       </c>
     </row>
@@ -66299,7 +66299,7 @@
       <c r="AD811" s="2" t="inlineStr"/>
       <c r="AE811" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01784; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01784</t>
         </is>
       </c>
     </row>
@@ -66372,7 +66372,7 @@
       <c r="AD812" s="2" t="inlineStr"/>
       <c r="AE812" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01710; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01710</t>
         </is>
       </c>
     </row>
@@ -66441,7 +66441,7 @@
       <c r="AD813" s="2" t="inlineStr"/>
       <c r="AE813" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00850; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00850</t>
         </is>
       </c>
     </row>
@@ -66514,7 +66514,7 @@
       <c r="AD814" s="2" t="inlineStr"/>
       <c r="AE814" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00510; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00510</t>
         </is>
       </c>
     </row>
@@ -66587,7 +66587,7 @@
       <c r="AD815" s="2" t="inlineStr"/>
       <c r="AE815" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00936; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00936</t>
         </is>
       </c>
     </row>
@@ -66660,7 +66660,7 @@
       <c r="AD816" s="2" t="inlineStr"/>
       <c r="AE816" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00906; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00906</t>
         </is>
       </c>
     </row>
@@ -66733,7 +66733,7 @@
       <c r="AD817" s="2" t="inlineStr"/>
       <c r="AE817" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01259; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01259</t>
         </is>
       </c>
     </row>
@@ -66806,7 +66806,7 @@
       <c r="AD818" s="2" t="inlineStr"/>
       <c r="AE818" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02037; no individual NPI â find clinic to enrich; NV lic #B01160; disciplinary action on record</t>
+          <t>NV lic #B02037</t>
         </is>
       </c>
     </row>
@@ -66879,7 +66879,7 @@
       <c r="AD819" s="2" t="inlineStr"/>
       <c r="AE819" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01775; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01775</t>
         </is>
       </c>
     </row>
@@ -66952,7 +66952,7 @@
       <c r="AD820" s="2" t="inlineStr"/>
       <c r="AE820" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01881; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01881</t>
         </is>
       </c>
     </row>
@@ -67025,7 +67025,7 @@
       <c r="AD821" s="2" t="inlineStr"/>
       <c r="AE821" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01713; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01713</t>
         </is>
       </c>
     </row>
@@ -67098,7 +67098,7 @@
       <c r="AD822" s="2" t="inlineStr"/>
       <c r="AE822" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01715; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01715</t>
         </is>
       </c>
     </row>
@@ -67171,7 +67171,7 @@
       <c r="AD823" s="2" t="inlineStr"/>
       <c r="AE823" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02142; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02142</t>
         </is>
       </c>
     </row>
@@ -67240,7 +67240,7 @@
       <c r="AD824" s="2" t="inlineStr"/>
       <c r="AE824" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01742; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01742</t>
         </is>
       </c>
     </row>
@@ -67309,7 +67309,7 @@
       <c r="AD825" s="2" t="inlineStr"/>
       <c r="AE825" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02131; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02131</t>
         </is>
       </c>
     </row>
@@ -67382,7 +67382,7 @@
       <c r="AD826" s="2" t="inlineStr"/>
       <c r="AE826" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01445; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01445</t>
         </is>
       </c>
     </row>
@@ -67451,7 +67451,7 @@
       <c r="AD827" s="2" t="inlineStr"/>
       <c r="AE827" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00601; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00601</t>
         </is>
       </c>
     </row>
@@ -67520,7 +67520,7 @@
       <c r="AD828" s="2" t="inlineStr"/>
       <c r="AE828" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01607; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01607</t>
         </is>
       </c>
     </row>
@@ -67593,7 +67593,7 @@
       <c r="AD829" s="2" t="inlineStr"/>
       <c r="AE829" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02110; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02110</t>
         </is>
       </c>
     </row>
@@ -67666,7 +67666,7 @@
       <c r="AD830" s="2" t="inlineStr"/>
       <c r="AE830" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01804; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01804</t>
         </is>
       </c>
     </row>
@@ -67739,7 +67739,7 @@
       <c r="AD831" s="2" t="inlineStr"/>
       <c r="AE831" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01767; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01767</t>
         </is>
       </c>
     </row>
@@ -67808,7 +67808,7 @@
       <c r="AD832" s="2" t="inlineStr"/>
       <c r="AE832" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02055; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02055</t>
         </is>
       </c>
     </row>
@@ -67881,7 +67881,7 @@
       <c r="AD833" s="2" t="inlineStr"/>
       <c r="AE833" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01952; no individual NPI â find clinic to enrich; NV lic #B00073</t>
+          <t>NV lic #B01952</t>
         </is>
       </c>
     </row>
@@ -67954,7 +67954,7 @@
       <c r="AD834" s="2" t="inlineStr"/>
       <c r="AE834" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01992; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01992</t>
         </is>
       </c>
     </row>
@@ -68023,7 +68023,7 @@
       <c r="AD835" s="2" t="inlineStr"/>
       <c r="AE835" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01470; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01470</t>
         </is>
       </c>
     </row>
@@ -68096,7 +68096,7 @@
       <c r="AD836" s="2" t="inlineStr"/>
       <c r="AE836" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01799; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01799</t>
         </is>
       </c>
     </row>
@@ -68165,7 +68165,7 @@
       <c r="AD837" s="2" t="inlineStr"/>
       <c r="AE837" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02082; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02082</t>
         </is>
       </c>
     </row>
@@ -68238,7 +68238,7 @@
       <c r="AD838" s="2" t="inlineStr"/>
       <c r="AE838" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01773; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01773</t>
         </is>
       </c>
     </row>
@@ -68311,7 +68311,7 @@
       <c r="AD839" s="2" t="inlineStr"/>
       <c r="AE839" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02058; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02058</t>
         </is>
       </c>
     </row>
@@ -68384,7 +68384,7 @@
       <c r="AD840" s="2" t="inlineStr"/>
       <c r="AE840" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01559; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01559</t>
         </is>
       </c>
     </row>
@@ -68457,7 +68457,7 @@
       <c r="AD841" s="2" t="inlineStr"/>
       <c r="AE841" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02148; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02148</t>
         </is>
       </c>
     </row>
@@ -68530,7 +68530,7 @@
       <c r="AD842" s="2" t="inlineStr"/>
       <c r="AE842" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01990; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01990</t>
         </is>
       </c>
     </row>
@@ -68599,7 +68599,7 @@
       <c r="AD843" s="2" t="inlineStr"/>
       <c r="AE843" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01909; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01909</t>
         </is>
       </c>
     </row>
@@ -68672,7 +68672,7 @@
       <c r="AD844" s="2" t="inlineStr"/>
       <c r="AE844" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02021; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02021</t>
         </is>
       </c>
     </row>
@@ -68745,7 +68745,7 @@
       <c r="AD845" s="2" t="inlineStr"/>
       <c r="AE845" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01964; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01964</t>
         </is>
       </c>
     </row>
@@ -68818,7 +68818,7 @@
       <c r="AD846" s="2" t="inlineStr"/>
       <c r="AE846" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02071; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02071</t>
         </is>
       </c>
     </row>
@@ -68891,7 +68891,7 @@
       <c r="AD847" s="2" t="inlineStr"/>
       <c r="AE847" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00650; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00650</t>
         </is>
       </c>
     </row>
@@ -68964,7 +68964,7 @@
       <c r="AD848" s="2" t="inlineStr"/>
       <c r="AE848" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02092; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02092</t>
         </is>
       </c>
     </row>
@@ -69037,7 +69037,7 @@
       <c r="AD849" s="2" t="inlineStr"/>
       <c r="AE849" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02111; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02111</t>
         </is>
       </c>
     </row>
@@ -69110,7 +69110,7 @@
       <c r="AD850" s="2" t="inlineStr"/>
       <c r="AE850" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01693; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01693</t>
         </is>
       </c>
     </row>
@@ -69183,7 +69183,7 @@
       <c r="AD851" s="2" t="inlineStr"/>
       <c r="AE851" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02107; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02107</t>
         </is>
       </c>
     </row>
@@ -69256,7 +69256,7 @@
       <c r="AD852" s="2" t="inlineStr"/>
       <c r="AE852" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01005; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01005</t>
         </is>
       </c>
     </row>
@@ -69329,7 +69329,7 @@
       <c r="AD853" s="2" t="inlineStr"/>
       <c r="AE853" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01577; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01577</t>
         </is>
       </c>
     </row>
@@ -69402,7 +69402,7 @@
       <c r="AD854" s="2" t="inlineStr"/>
       <c r="AE854" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01762; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01762</t>
         </is>
       </c>
     </row>
@@ -69471,7 +69471,7 @@
       <c r="AD855" s="2" t="inlineStr"/>
       <c r="AE855" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00955; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00955</t>
         </is>
       </c>
     </row>
@@ -69544,7 +69544,7 @@
       <c r="AD856" s="2" t="inlineStr"/>
       <c r="AE856" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01903; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01903</t>
         </is>
       </c>
     </row>
@@ -69617,7 +69617,7 @@
       <c r="AD857" s="2" t="inlineStr"/>
       <c r="AE857" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01913; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01913</t>
         </is>
       </c>
     </row>
@@ -69686,7 +69686,7 @@
       <c r="AD858" s="2" t="inlineStr"/>
       <c r="AE858" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01872; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01872</t>
         </is>
       </c>
     </row>
@@ -69759,7 +69759,7 @@
       <c r="AD859" s="2" t="inlineStr"/>
       <c r="AE859" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02137; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02137</t>
         </is>
       </c>
     </row>
@@ -69832,7 +69832,7 @@
       <c r="AD860" s="2" t="inlineStr"/>
       <c r="AE860" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00885; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00885</t>
         </is>
       </c>
     </row>
@@ -69905,7 +69905,7 @@
       <c r="AD861" s="2" t="inlineStr"/>
       <c r="AE861" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02100; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02100</t>
         </is>
       </c>
     </row>
@@ -69978,7 +69978,7 @@
       <c r="AD862" s="2" t="inlineStr"/>
       <c r="AE862" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00899; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00899</t>
         </is>
       </c>
     </row>
@@ -70047,7 +70047,7 @@
       <c r="AD863" s="2" t="inlineStr"/>
       <c r="AE863" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01514; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01514</t>
         </is>
       </c>
     </row>
@@ -70120,7 +70120,7 @@
       <c r="AD864" s="2" t="inlineStr"/>
       <c r="AE864" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02164; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02164</t>
         </is>
       </c>
     </row>
@@ -70193,7 +70193,7 @@
       <c r="AD865" s="2" t="inlineStr"/>
       <c r="AE865" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01522; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01522</t>
         </is>
       </c>
     </row>
@@ -70266,7 +70266,7 @@
       <c r="AD866" s="2" t="inlineStr"/>
       <c r="AE866" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02091; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02091</t>
         </is>
       </c>
     </row>
@@ -70339,7 +70339,7 @@
       <c r="AD867" s="2" t="inlineStr"/>
       <c r="AE867" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01061; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01061</t>
         </is>
       </c>
     </row>
@@ -70412,7 +70412,7 @@
       <c r="AD868" s="2" t="inlineStr"/>
       <c r="AE868" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01796; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01796</t>
         </is>
       </c>
     </row>
@@ -70485,7 +70485,7 @@
       <c r="AD869" s="2" t="inlineStr"/>
       <c r="AE869" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02139; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02139</t>
         </is>
       </c>
     </row>
@@ -70558,7 +70558,7 @@
       <c r="AD870" s="2" t="inlineStr"/>
       <c r="AE870" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02150; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02150</t>
         </is>
       </c>
     </row>
@@ -70631,7 +70631,7 @@
       <c r="AD871" s="2" t="inlineStr"/>
       <c r="AE871" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B00712; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B00712</t>
         </is>
       </c>
     </row>
@@ -70700,7 +70700,7 @@
       <c r="AD872" s="2" t="inlineStr"/>
       <c r="AE872" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01611; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01611</t>
         </is>
       </c>
     </row>
@@ -70773,7 +70773,7 @@
       <c r="AD873" s="2" t="inlineStr"/>
       <c r="AE873" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01803; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01803</t>
         </is>
       </c>
     </row>
@@ -70846,7 +70846,7 @@
       <c r="AD874" s="2" t="inlineStr"/>
       <c r="AE874" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02073; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02073</t>
         </is>
       </c>
     </row>
@@ -70915,7 +70915,7 @@
       <c r="AD875" s="2" t="inlineStr"/>
       <c r="AE875" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01919; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01919</t>
         </is>
       </c>
     </row>
@@ -70988,7 +70988,7 @@
       <c r="AD876" s="2" t="inlineStr"/>
       <c r="AE876" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01069; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01069</t>
         </is>
       </c>
     </row>
@@ -71057,7 +71057,7 @@
       <c r="AD877" s="2" t="inlineStr"/>
       <c r="AE877" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B01935; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B01935</t>
         </is>
       </c>
     </row>
@@ -71130,7 +71130,7 @@
       <c r="AD878" s="2" t="inlineStr"/>
       <c r="AE878" s="2" t="inlineStr">
         <is>
-          <t>NV lic #B02038; no individual NPI â find clinic to enrich</t>
+          <t>NV lic #B02038</t>
         </is>
       </c>
     </row>

</xml_diff>